<commit_message>
update the test11 and 12
</commit_message>
<xml_diff>
--- a/boltz_experiment_master.xlsx
+++ b/boltz_experiment_master.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/39b8f5b1ceed89e2/Desktop/MSc_research/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="83" documentId="8_{5F9DF5E2-6C68-4678-AFC6-E59FBBEA935A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CFDC983C-4944-495A-A4CD-9F1A5D9D7D54}"/>
+  <xr:revisionPtr revIDLastSave="104" documentId="8_{5F9DF5E2-6C68-4678-AFC6-E59FBBEA935A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{61052453-9BF3-4352-BA6B-7CE583620FEB}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{B693CC76-476B-46BE-908F-567C50EF84D4}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="95">
   <si>
     <t>Experiment ID</t>
   </si>
@@ -352,13 +352,74 @@
   <si>
     <t>Twenty lipids were successfully added to the protein, which means we can proceed with running the full pipeline on the HPC system.</t>
     <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>011</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>HPC: Boltz2/Biopython/OpenMM</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>010_3_fgfr2_minimized.pdb</t>
+  </si>
+  <si>
+    <t>straighten the linker between the TM and ICD/ECD regions using Biopython</t>
+  </si>
+  <si>
+    <t>011_3_fgfr2_clean_minimized.pdb</t>
+  </si>
+  <si>
+    <t>OpenMM successfully minimized the energy after straightening the linker, but the linker between the TM and ICD does not appear reasonable based on UniProt information.</t>
+  </si>
+  <si>
+    <t>012</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>use the Boltz2 prediction model generated in the test10</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>fine</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Tahoma"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t>‑</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="新細明體"/>
+        <family val="2"/>
+        <charset val="136"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>tune the linker between the TM and ICD and separate it from the ICD domain</t>
+    </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>012_3_fgfr2_clean_minimized.pdb</t>
+  </si>
+  <si>
+    <t>The conformation appears physically reasonable at this stage.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -391,6 +452,13 @@
       <family val="2"/>
       <charset val="136"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -781,7 +849,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{155A3948-C683-4751-821F-C1EF1E91D33B}">
-  <dimension ref="A1:L11"/>
+  <dimension ref="A1:L13"/>
   <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="13.81640625" style="1" bestFit="1" customWidth="1"/>
@@ -792,7 +860,7 @@
     <col min="6" max="6" width="12.81640625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="12.1796875" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="19.36328125" customWidth="1"/>
-    <col min="9" max="9" width="10.26953125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="18.6328125" customWidth="1"/>
     <col min="10" max="10" width="15.08984375" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="15.08984375" customWidth="1"/>
     <col min="12" max="12" width="18" bestFit="1" customWidth="1"/>
@@ -1203,6 +1271,9 @@
       <c r="H11" t="s">
         <v>81</v>
       </c>
+      <c r="I11" t="s">
+        <v>86</v>
+      </c>
       <c r="J11" t="s">
         <v>23</v>
       </c>
@@ -1211,6 +1282,82 @@
       </c>
       <c r="L11" t="s">
         <v>83</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.4">
+      <c r="A12" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="B12" t="s">
+        <v>91</v>
+      </c>
+      <c r="C12" t="s">
+        <v>16</v>
+      </c>
+      <c r="D12" t="s">
+        <v>18</v>
+      </c>
+      <c r="E12" t="s">
+        <v>19</v>
+      </c>
+      <c r="F12" t="s">
+        <v>20</v>
+      </c>
+      <c r="G12" t="s">
+        <v>21</v>
+      </c>
+      <c r="H12" t="s">
+        <v>87</v>
+      </c>
+      <c r="I12" t="s">
+        <v>88</v>
+      </c>
+      <c r="J12" t="s">
+        <v>23</v>
+      </c>
+      <c r="K12" t="s">
+        <v>85</v>
+      </c>
+      <c r="L12" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.4">
+      <c r="A13" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B13" t="s">
+        <v>91</v>
+      </c>
+      <c r="C13" t="s">
+        <v>16</v>
+      </c>
+      <c r="D13" t="s">
+        <v>18</v>
+      </c>
+      <c r="E13" t="s">
+        <v>19</v>
+      </c>
+      <c r="F13" t="s">
+        <v>20</v>
+      </c>
+      <c r="G13" t="s">
+        <v>21</v>
+      </c>
+      <c r="H13" t="s">
+        <v>92</v>
+      </c>
+      <c r="I13" t="s">
+        <v>93</v>
+      </c>
+      <c r="J13" t="s">
+        <v>23</v>
+      </c>
+      <c r="K13" t="s">
+        <v>85</v>
+      </c>
+      <c r="L13" t="s">
+        <v>94</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update the test 13
</commit_message>
<xml_diff>
--- a/boltz_experiment_master.xlsx
+++ b/boltz_experiment_master.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/39b8f5b1ceed89e2/Desktop/MSc_research/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="104" documentId="8_{5F9DF5E2-6C68-4678-AFC6-E59FBBEA935A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{61052453-9BF3-4352-BA6B-7CE583620FEB}"/>
+  <xr:revisionPtr revIDLastSave="113" documentId="8_{5F9DF5E2-6C68-4678-AFC6-E59FBBEA935A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0C18D347-04D4-492C-9B72-EB6A182CC82C}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{B693CC76-476B-46BE-908F-567C50EF84D4}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="100">
   <si>
     <t>Experiment ID</t>
   </si>
@@ -413,6 +413,49 @@
   </si>
   <si>
     <t>The conformation appears physically reasonable at this stage.</t>
+  </si>
+  <si>
+    <t>013</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Compiling all pipeline steps in Nextflow</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>013_3_fgfr2_clean_minimized.pdb</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>HPC: NextFlow (Boltz2/ChimeraX/Biopython/OpenMM)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>Overall, although the conformation in Test 13 is not as well</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Tahoma"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t>‑</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="新細明體"/>
+        <family val="2"/>
+        <charset val="136"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>refined as that in Test 12, it remains acceptable for downstream analysis and is sufficient for executing the entire pipeline through a single Nextflow script.</t>
+    </r>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -849,7 +892,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{155A3948-C683-4751-821F-C1EF1E91D33B}">
-  <dimension ref="A1:L13"/>
+  <dimension ref="A1:L14"/>
   <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="13.81640625" style="1" bestFit="1" customWidth="1"/>
@@ -1358,6 +1401,44 @@
       </c>
       <c r="L13" t="s">
         <v>94</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.4">
+      <c r="A14" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B14" t="s">
+        <v>80</v>
+      </c>
+      <c r="C14" t="s">
+        <v>16</v>
+      </c>
+      <c r="D14" t="s">
+        <v>18</v>
+      </c>
+      <c r="E14" t="s">
+        <v>19</v>
+      </c>
+      <c r="F14" t="s">
+        <v>20</v>
+      </c>
+      <c r="G14" t="s">
+        <v>21</v>
+      </c>
+      <c r="H14" t="s">
+        <v>96</v>
+      </c>
+      <c r="I14" t="s">
+        <v>97</v>
+      </c>
+      <c r="J14" t="s">
+        <v>23</v>
+      </c>
+      <c r="K14" t="s">
+        <v>98</v>
+      </c>
+      <c r="L14" t="s">
+        <v>99</v>
       </c>
     </row>
   </sheetData>

</xml_diff>